<commit_message>
Cambios En la tarifa-Inflacion
</commit_message>
<xml_diff>
--- a/bitacora_web_avance/plantilla/plantilla_tarifas.xlsx
+++ b/bitacora_web_avance/plantilla/plantilla_tarifas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0076A05-99DA-440C-B35E-035C9A428E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E30ABB25-05D4-4E43-AAF5-4E5FE4FF9955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{BE96FE0C-B884-44D3-89DB-E867C57A1353}"/>
+    <workbookView xWindow="4428" yWindow="1620" windowWidth="17280" windowHeight="9960" xr2:uid="{3BF71119-C2EE-485A-9C09-4A4F49E6BC5A}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -35,45 +35,48 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>AUTORIDAD PORTUARIA DE MANTA</t>
   </si>
   <si>
+    <t>DPTO. DE OPERACIONES - TERMINAL PESQUERO Y CABOTAJE</t>
+  </si>
+  <si>
     <t>REPORTE TARIFA</t>
   </si>
   <si>
-    <t>DPTO. DE OPERACIONES - TERMINAL PESQUERO Y CABOTAJE</t>
-  </si>
-  <si>
     <t>Fecha de Emisión:</t>
   </si>
   <si>
+    <t>TASA</t>
+  </si>
+  <si>
+    <t>COD.TARIFA</t>
+  </si>
+  <si>
+    <t>TARIFA</t>
+  </si>
+  <si>
     <t>VALOR</t>
   </si>
   <si>
     <t>FORMULA</t>
   </si>
   <si>
+    <t>INFLACION</t>
+  </si>
+  <si>
     <t>DETALLE</t>
   </si>
   <si>
-    <t>TARIFA</t>
-  </si>
-  <si>
-    <t>COD.TARIFA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     COD,PARTIDA</t>
+    <t xml:space="preserve">     COD.PARTIDA</t>
   </si>
   <si>
     <t>PARTIDA</t>
   </si>
   <si>
-    <t>INFLACION</t>
-  </si>
-  <si>
-    <t>TASA</t>
+    <t>ESTADO</t>
   </si>
 </sst>
 </file>
@@ -97,6 +100,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF00286C"/>
@@ -112,14 +123,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -130,7 +133,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -142,7 +145,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -174,28 +177,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -230,10 +232,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F907048A-1720-C584-E6D5-62224CA0C978}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DD73C64B-252D-4550-8690-18EE7CA0651B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -564,260 +566,133 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{109E6963-B780-4C5F-B6EB-8C82D748515C}">
-  <dimension ref="A1:K28"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E96124A7-4B3D-457D-85F1-175974DA25AF}">
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="26.44140625" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" customWidth="1"/>
-    <col min="5" max="5" width="31" customWidth="1"/>
-    <col min="6" max="6" width="24.33203125" customWidth="1"/>
-    <col min="7" max="7" width="24.88671875" customWidth="1"/>
-    <col min="8" max="8" width="23.109375" customWidth="1"/>
-    <col min="9" max="9" width="33.88671875" customWidth="1"/>
+    <col min="1" max="1" width="23.21875" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" customWidth="1"/>
+    <col min="3" max="3" width="25.109375" customWidth="1"/>
+    <col min="4" max="4" width="13.21875" customWidth="1"/>
+    <col min="5" max="5" width="23" customWidth="1"/>
+    <col min="6" max="6" width="23.21875" customWidth="1"/>
+    <col min="7" max="7" width="25" customWidth="1"/>
+    <col min="8" max="8" width="20.5546875" customWidth="1"/>
+    <col min="9" max="9" width="36" customWidth="1"/>
+    <col min="10" max="10" width="18.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G6" s="3"/>
+      <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>10</v>
+      <c r="J7" s="7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E28" s="3"/>
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>